<commit_message>
feat: add test plan and update documentation for distributing total acres feature on iOS
</commit_message>
<xml_diff>
--- a/playwright/test-plans/authenticated/work-orders-distribute-acres-ios.xlsx
+++ b/playwright/test-plans/authenticated/work-orders-distribute-acres-ios.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Test Data" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Cases'!$A$5:$N$45</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Cases'!$A$5:$N$44</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="260">
   <si>
     <t xml:space="preserve">ADO #25969 — Distribute Total Acres Equally Across Selected Users (iOS) — Test Cases</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: ADO #25969 + product answers 2026-10-09 (all WO types except Inspection; multiple resources, Individual default; overdue allowed) + developer handover notes (branch bugfix/25969-…, commit ad8056e5b). Plan: playwright/test-plans/authenticated/work-orders-distribute-acres-ios.md. No PSD or mock-up attached to the ticket.</t>
+    <t xml:space="preserve">Source: ADO #25969 + product answers 2026-10-09 (all WO types except Inspection; multiple resources, Individual default; overdue allowed; iOS + web only, no D365 acreage posting) + developer handover notes (branch bugfix/25969-…, commit ad8056e5b). Plan: playwright/test-plans/authenticated/work-orders-distribute-acres-ios.md. No PSD or mock-up attached to the ticket.</t>
   </si>
   <si>
     <t xml:space="preserve">Legend: fill in the yellow Result column (Pass / Fail / Blocked / Not Run) and the Run details cells on the Summary tab. Example: DIST-012 — 4.75 acres across 2 users must show 2.37 and 2.38. Notes flag product-confirmed and still-open behaviour.</t>
@@ -448,10 +448,10 @@
     <t xml:space="preserve">After DIST-031, open WO A on QA web → View → Plots grid and View Spent Hours</t>
   </si>
   <si>
-    <t xml:space="preserve">Plot progress / area includes the 10.00 total. Per-user split matches mobile. Nothing posts to D365 at this point</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Web labels (Plots grid / View Spent Hours) to be confirmed on first run.</t>
+    <t xml:space="preserve">Plot progress / area includes the 10.00 total. Per-user split matches mobile. Acreage is not posted to D365, so there is nothing to check there</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web labels (Plots grid / View Spent Hours) to be confirmed on first run. No D365 posting of acreage (product 2026-10-09).</t>
   </si>
   <si>
     <t xml:space="preserve">DIST-034</t>
@@ -589,18 +589,6 @@
     <t xml:space="preserve">Product says all types except Inspection. Dev notes say this screen has no per-user area. Record what shows and confirm with product before filing</t>
   </si>
   <si>
-    <t xml:space="preserve">DIST-055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finops app</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iOS build with commit ad8056e5b; logged in on mobile as a Supervisor (VBS tenant, QA env). Finops app installed, same user</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open the equivalent screen in the Finops app</t>
-  </si>
-  <si>
     <t xml:space="preserve">DIST-056</t>
   </si>
   <si>
@@ -805,7 +793,10 @@
     <t xml:space="preserve">2. Display: shown only with multiple resources. Default view is always Individual, so the mode is not remembered (DIST-001, DIST-005, DIST-051).</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Overdue allowed: yes. Read as Total Acres above the block's remaining area (DIST-019). Overdue WOs past their End Date are also covered (DIST-057). Confirm which one product meant.</t>
+    <t xml:space="preserve">3. Platforms: iOS and web only. Acreage is not posted to D365 (DIST-033).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Overdue allowed: yes. Read as Total Acres above the block's remaining area (DIST-019). Overdue WOs past their End Date are also covered (DIST-057). Confirm which one product meant.</t>
   </si>
   <si>
     <t xml:space="preserve">Open questions for product</t>
@@ -1324,7 +1315,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2847,7 +2838,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
         <v>186</v>
       </c>
@@ -2864,10 +2855,10 @@
         <v>21</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="H40" s="4" t="s">
         <v>188</v>
@@ -2877,22 +2868,24 @@
       </c>
       <c r="J40" s="4"/>
       <c r="K40" s="4" t="s">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="L40" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M40" s="4"/>
+        <v>27</v>
+      </c>
+      <c r="M40" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="N40" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>161</v>
@@ -2904,20 +2897,20 @@
         <v>21</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="G41" s="4" t="s">
         <v>32</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J41" s="4"/>
       <c r="K41" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="L41" s="4" t="s">
         <v>27</v>
@@ -2929,15 +2922,15 @@
         <v>29</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>161</v>
+        <v>198</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>20</v>
@@ -2949,52 +2942,50 @@
         <v>43</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="J42" s="4"/>
       <c r="K42" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="L42" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="M42" s="4"/>
+      <c r="N42" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G43" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="L42" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="M42" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="N42" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="G43" s="4" t="s">
-        <v>203</v>
-      </c>
       <c r="H43" s="4" t="s">
-        <v>204</v>
+        <v>24</v>
       </c>
       <c r="I43" s="4" t="s">
         <v>205</v>
@@ -3019,7 +3010,7 @@
         <v>208</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>20</v>
@@ -3031,7 +3022,7 @@
         <v>48</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="H44" s="4" t="s">
         <v>24</v>
@@ -3046,61 +3037,21 @@
       <c r="L44" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M44" s="4"/>
+      <c r="M44" s="4" t="s">
+        <v>211</v>
+      </c>
       <c r="N44" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="G45" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="H45" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I45" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="J45" s="4"/>
-      <c r="K45" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="L45" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M45" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="N45" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:N45"/>
+  <autoFilter ref="A5:N44"/>
   <mergeCells count="3">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A3:N3"/>
   </mergeCells>
-  <conditionalFormatting sqref="N6:N45">
+  <conditionalFormatting sqref="N6:N44">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3112,7 +3063,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N6:N45" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N6:N44" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3142,41 +3093,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B4" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$N$6:$N$45,"Pass")</f>
+        <f aca="false">COUNTIF('Test Cases'!$N$6:$N$44,"Pass")</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B5" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$N$6:$N$45,"Fail")</f>
+        <f aca="false">COUNTIF('Test Cases'!$N$6:$N$44,"Fail")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B6" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$N$6:$N$45,"Blocked")</f>
+        <f aca="false">COUNTIF('Test Cases'!$N$6:$N$44,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -3185,25 +3136,25 @@
         <v>29</v>
       </c>
       <c r="B7" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$N$6:$N$45,"Not Run")</f>
-        <v>40</v>
+        <f aca="false">COUNTIF('Test Cases'!$N$6:$N$44,"Not Run")</f>
+        <v>39</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3211,7 +3162,7 @@
         <v>22</v>
       </c>
       <c r="B11" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$F$6:$F$45,"P1")</f>
+        <f aca="false">COUNTIF('Test Cases'!$F$6:$F$44,"P1")</f>
         <v>22</v>
       </c>
     </row>
@@ -3220,7 +3171,7 @@
         <v>43</v>
       </c>
       <c r="B12" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$F$6:$F$45,"P2")</f>
+        <f aca="false">COUNTIF('Test Cases'!$F$6:$F$44,"P2")</f>
         <v>14</v>
       </c>
     </row>
@@ -3229,25 +3180,25 @@
         <v>48</v>
       </c>
       <c r="B13" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$F$6:$F$45,"P3")</f>
-        <v>4</v>
+        <f aca="false">COUNTIF('Test Cases'!$F$6:$F$44,"P3")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B14" s="7" t="n">
         <f aca="false">SUM(B11:B13)</f>
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3255,7 +3206,7 @@
         <v>19</v>
       </c>
       <c r="B17" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$45,"Display and default")</f>
+        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Display and default")</f>
         <v>5</v>
       </c>
     </row>
@@ -3264,7 +3215,7 @@
         <v>53</v>
       </c>
       <c r="B18" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$45,"Distribution and rounding (Distribute equally)")</f>
+        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Distribution and rounding (Distribute equally)")</f>
         <v>10</v>
       </c>
     </row>
@@ -3273,7 +3224,7 @@
         <v>99</v>
       </c>
       <c r="B19" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$45,"Selection changes")</f>
+        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Selection changes")</f>
         <v>6</v>
       </c>
     </row>
@@ -3282,7 +3233,7 @@
         <v>124</v>
       </c>
       <c r="B20" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$45,"Switching back and saving")</f>
+        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Switching back and saving")</f>
         <v>5</v>
       </c>
     </row>
@@ -3291,7 +3242,7 @@
         <v>147</v>
       </c>
       <c r="B21" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$45,"Multi-block End Job")</f>
+        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Multi-block End Job")</f>
         <v>3</v>
       </c>
     </row>
@@ -3300,54 +3251,54 @@
         <v>161</v>
       </c>
       <c r="B22" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$45,"Work order type coverage")</f>
-        <v>8</v>
+        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Work order type coverage")</f>
+        <v>7</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B23" s="8" t="n">
-        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$45,"UI and language")</f>
+        <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"UI and language")</f>
         <v>3</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B24" s="7" t="n">
         <f aca="false">SUM(B17:B23)</f>
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B30" s="9"/>
     </row>
@@ -3367,7 +3318,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -3376,159 +3327,166 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="B19" s="12"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
-        <v>260</v>
-      </c>
-      <c r="B22" s="12"/>
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="B20" s="12"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="B24" s="12"/>
     </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="B25" s="12"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A20:B20"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
fix: update workbook filename in test plan and refine product answers in work item
</commit_message>
<xml_diff>
--- a/playwright/test-plans/authenticated/work-orders-distribute-acres-ios.xlsx
+++ b/playwright/test-plans/authenticated/work-orders-distribute-acres-ios.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="253">
   <si>
     <t xml:space="preserve">ADO #25969 — Distribute Total Acres Equally Across Selected Users (iOS) — Test Cases</t>
   </si>
@@ -508,30 +508,15 @@
     <t xml:space="preserve">Block 1 still in Distribute equally with the same total and shares</t>
   </si>
   <si>
-    <t xml:space="preserve">DIST-050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rows/beds block: hidden</t>
+    <t xml:space="preserve">DIST-051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single-resource block: hidden</t>
   </si>
   <si>
     <t xml:space="preserve">Work order type coverage</t>
   </si>
   <si>
-    <t xml:space="preserve">iOS build with commit ad8056e5b; logged in on mobile as a Supervisor (VBS tenant, QA env). WO C: rows/beds block, 2+ users</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO C → Pause Job → Progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No switch. Rows/beds entry as before</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIST-051</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Single-resource block: hidden</t>
-  </si>
-  <si>
     <t xml:space="preserve">iOS build with commit ad8056e5b; logged in on mobile as a Supervisor (VBS tenant, QA env). WO D: area-based block, 1 resource only</t>
   </si>
   <si>
@@ -740,12 +725,6 @@
   </si>
   <si>
     <t xml:space="preserve">Same as A but with 2 blocks (for multi-block End Job)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WO C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planned WO with a rows/beds block and 2+ users (regression)</t>
   </si>
   <si>
     <t xml:space="preserve">WO D</t>
@@ -952,12 +931,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -977,23 +960,23 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1005,6 +988,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1014,7 +1001,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1026,6 +1013,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1318,1732 +1313,1693 @@
   <dimension ref="A1:N44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="L5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="N5" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="4" t="s">
+      <c r="D6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4" t="s">
+      <c r="J6" s="5"/>
+      <c r="K6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="L6" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="M6" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="N6" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="N6" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="4" t="s">
+      <c r="D7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4" t="s">
+      <c r="J7" s="5"/>
+      <c r="K7" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L7" s="4" t="s">
+      <c r="L7" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M7" s="4"/>
-      <c r="N7" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="M7" s="5"/>
+      <c r="N7" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="4" t="s">
+      <c r="D8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4" t="s">
+      <c r="J8" s="5"/>
+      <c r="K8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="L8" s="4" t="s">
+      <c r="L8" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M8" s="4"/>
-      <c r="N8" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="M8" s="5"/>
+      <c r="N8" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" s="4" t="s">
+      <c r="D9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4" t="s">
+      <c r="J9" s="5"/>
+      <c r="K9" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="L9" s="4" t="s">
+      <c r="L9" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M9" s="4"/>
-      <c r="N9" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="M9" s="5"/>
+      <c r="N9" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" s="4" t="s">
+      <c r="D10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4" t="s">
+      <c r="J10" s="5"/>
+      <c r="K10" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="L10" s="4" t="s">
+      <c r="L10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="M10" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="N10" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="N10" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="4" t="s">
+      <c r="D11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="L11" s="4" t="s">
+      <c r="L11" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M11" s="4"/>
-      <c r="N11" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="M11" s="5"/>
+      <c r="N11" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="D12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="J12" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="K12" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="L12" s="4" t="s">
+      <c r="L12" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="N12" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="N12" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F13" s="4" t="s">
+      <c r="D13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J13" s="4" t="s">
+      <c r="J13" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="K13" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="L13" s="4" t="s">
+      <c r="L13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M13" s="4" t="s">
+      <c r="M13" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="N13" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="N13" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F14" s="4" t="s">
+      <c r="D14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="J14" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="K14" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="L14" s="4" t="s">
+      <c r="L14" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M14" s="4" t="s">
+      <c r="M14" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="N14" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="N14" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F15" s="4" t="s">
+      <c r="D15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H15" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J15" s="4" t="s">
+      <c r="J15" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="K15" s="4" t="s">
+      <c r="K15" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="L15" s="4" t="s">
+      <c r="L15" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M15" s="4" t="s">
+      <c r="M15" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="N15" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="N15" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F16" s="4" t="s">
+      <c r="D16" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="J16" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="K16" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="L16" s="4" t="s">
+      <c r="L16" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M16" s="4" t="s">
+      <c r="M16" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="N16" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="N16" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F17" s="4" t="s">
+      <c r="D17" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="H17" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J17" s="4" t="s">
+      <c r="J17" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="K17" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="L17" s="4" t="s">
+      <c r="L17" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M17" s="4"/>
-      <c r="N17" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="M17" s="5"/>
+      <c r="N17" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F18" s="4" t="s">
+      <c r="D18" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="J18" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="K18" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="L18" s="4" t="s">
+      <c r="L18" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M18" s="4"/>
-      <c r="N18" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="M18" s="5"/>
+      <c r="N18" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F19" s="4" t="s">
+      <c r="D19" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="J19" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="K19" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="L19" s="4" t="s">
+      <c r="L19" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M19" s="4"/>
-      <c r="N19" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="M19" s="5"/>
+      <c r="N19" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F20" s="4" t="s">
+      <c r="D20" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F20" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H20" s="4" t="s">
+      <c r="H20" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="I20" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J20" s="4" t="s">
+      <c r="J20" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="K20" s="4" t="s">
+      <c r="K20" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="L20" s="4" t="s">
+      <c r="L20" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="M20" s="4" t="s">
+      <c r="M20" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="N20" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="N20" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F21" s="4" t="s">
+      <c r="D21" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F21" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H21" s="4" t="s">
+      <c r="H21" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I21" s="4" t="s">
+      <c r="I21" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4" t="s">
+      <c r="J21" s="5"/>
+      <c r="K21" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="L21" s="4" t="s">
+      <c r="L21" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M21" s="4"/>
-      <c r="N21" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="M21" s="5"/>
+      <c r="N21" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F22" s="4" t="s">
+      <c r="D22" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="I22" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4" t="s">
+      <c r="J22" s="5"/>
+      <c r="K22" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="L22" s="4" t="s">
+      <c r="L22" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M22" s="4"/>
-      <c r="N22" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="M22" s="5"/>
+      <c r="N22" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F23" s="4" t="s">
+      <c r="D23" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I23" s="4" t="s">
+      <c r="I23" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4" t="s">
+      <c r="J23" s="5"/>
+      <c r="K23" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="L23" s="4" t="s">
+      <c r="L23" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M23" s="4"/>
-      <c r="N23" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="M23" s="5"/>
+      <c r="N23" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F24" s="4" t="s">
+      <c r="D24" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="I24" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4" t="s">
+      <c r="J24" s="5"/>
+      <c r="K24" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="L24" s="4" t="s">
+      <c r="L24" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M24" s="4"/>
-      <c r="N24" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+      <c r="M24" s="5"/>
+      <c r="N24" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D25" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F25" s="4" t="s">
+      <c r="D25" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="H25" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I25" s="4" t="s">
+      <c r="I25" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4" t="s">
+      <c r="J25" s="5"/>
+      <c r="K25" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="L25" s="4" t="s">
+      <c r="L25" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M25" s="4"/>
-      <c r="N25" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="M25" s="5"/>
+      <c r="N25" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F26" s="4" t="s">
+      <c r="D26" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H26" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I26" s="4" t="s">
+      <c r="I26" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4" t="s">
+      <c r="J26" s="5"/>
+      <c r="K26" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="L26" s="4" t="s">
+      <c r="L26" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M26" s="4"/>
-      <c r="N26" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="M26" s="5"/>
+      <c r="N26" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D27" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F27" s="4" t="s">
+      <c r="D27" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F27" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="H27" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I27" s="4" t="s">
+      <c r="I27" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4" t="s">
+      <c r="J27" s="5"/>
+      <c r="K27" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="L27" s="4" t="s">
+      <c r="L27" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M27" s="4"/>
-      <c r="N27" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="M27" s="5"/>
+      <c r="N27" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F28" s="4" t="s">
+      <c r="D28" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="H28" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I28" s="4" t="s">
+      <c r="I28" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4" t="s">
+      <c r="J28" s="5"/>
+      <c r="K28" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="L28" s="4" t="s">
+      <c r="L28" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M28" s="4"/>
-      <c r="N28" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
+      <c r="M28" s="5"/>
+      <c r="N28" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D29" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F29" s="4" t="s">
+      <c r="D29" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F29" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G29" s="4" t="s">
+      <c r="G29" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H29" s="4" t="s">
+      <c r="H29" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I29" s="4" t="s">
+      <c r="I29" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4" t="s">
+      <c r="J29" s="5"/>
+      <c r="K29" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="L29" s="4" t="s">
+      <c r="L29" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M29" s="4"/>
-      <c r="N29" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="M29" s="5"/>
+      <c r="N29" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D30" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E30" s="4" t="s">
+      <c r="D30" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="G30" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H30" s="4" t="s">
+      <c r="H30" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I30" s="4" t="s">
+      <c r="I30" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4" t="s">
+      <c r="J30" s="5"/>
+      <c r="K30" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="L30" s="4" t="s">
+      <c r="L30" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M30" s="4" t="s">
+      <c r="M30" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="N30" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="N30" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D31" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F31" s="4" t="s">
+      <c r="D31" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F31" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="G31" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H31" s="4" t="s">
+      <c r="H31" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I31" s="4" t="s">
+      <c r="I31" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4" t="s">
+      <c r="J31" s="5"/>
+      <c r="K31" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="L31" s="4" t="s">
+      <c r="L31" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M31" s="4"/>
-      <c r="N31" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="M31" s="5"/>
+      <c r="N31" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D32" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F32" s="4" t="s">
+      <c r="D32" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G32" s="4" t="s">
+      <c r="G32" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H32" s="4" t="s">
+      <c r="H32" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="I32" s="4" t="s">
+      <c r="I32" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4" t="s">
+      <c r="J32" s="5"/>
+      <c r="K32" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="L32" s="4" t="s">
+      <c r="L32" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M32" s="4"/>
-      <c r="N32" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+      <c r="M32" s="5"/>
+      <c r="N32" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D33" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F33" s="4" t="s">
+      <c r="D33" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F33" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G33" s="4" t="s">
+      <c r="G33" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H33" s="4" t="s">
+      <c r="H33" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="I33" s="4" t="s">
+      <c r="I33" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4" t="s">
+      <c r="J33" s="5"/>
+      <c r="K33" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="L33" s="4" t="s">
+      <c r="L33" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M33" s="4"/>
-      <c r="N33" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="M33" s="5"/>
+      <c r="N33" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D34" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F34" s="4" t="s">
+      <c r="D34" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F34" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="G34" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H34" s="4" t="s">
+      <c r="H34" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="I34" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4" t="s">
+      <c r="J34" s="5"/>
+      <c r="K34" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="L34" s="4" t="s">
+      <c r="L34" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M34" s="4"/>
-      <c r="N34" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="M34" s="5"/>
+      <c r="N34" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="D35" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F35" s="4" t="s">
+      <c r="D35" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="G35" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H35" s="4" t="s">
+      <c r="H35" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="I35" s="4" t="s">
+      <c r="I35" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4" t="s">
+      <c r="J35" s="5"/>
+      <c r="K35" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="L35" s="4" t="s">
+      <c r="L35" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N35" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="L36" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="M36" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N36" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="L37" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="M37" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="N37" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="L38" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="M38" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="N38" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="I39" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="J39" s="5"/>
+      <c r="K39" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="L39" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="M39" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N39" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="I40" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="J40" s="5"/>
+      <c r="K40" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="L40" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="M40" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N40" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="H41" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="I41" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="J41" s="5"/>
+      <c r="K41" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="L41" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M35" s="4"/>
-      <c r="N35" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H36" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="I36" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="J36" s="4"/>
-      <c r="K36" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="L36" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="M36" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="N36" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H37" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="I37" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="L37" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="M37" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="N37" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H38" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="I38" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="J38" s="4"/>
-      <c r="K38" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="L38" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="M38" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="N38" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="G39" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H39" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="I39" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="J39" s="4"/>
-      <c r="K39" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="L39" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="M39" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="N39" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F40" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G40" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H40" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="I40" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="J40" s="4"/>
-      <c r="K40" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="L40" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="M40" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="N40" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H41" s="4" t="s">
+      <c r="M41" s="5"/>
+      <c r="N41" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="I41" s="4" t="s">
+      <c r="D42" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G42" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="J41" s="4"/>
-      <c r="K41" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="L41" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="M41" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="N41" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F42" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="G42" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="H42" s="4" t="s">
+      <c r="H42" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I42" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="I42" s="4" t="s">
+      <c r="J42" s="5"/>
+      <c r="K42" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="J42" s="4"/>
-      <c r="K42" s="4" t="s">
+      <c r="L42" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="M42" s="5"/>
+      <c r="N42" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="L42" s="4" t="s">
+      <c r="B43" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I43" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="J43" s="5"/>
+      <c r="K43" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="L43" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="M42" s="4"/>
-      <c r="N42" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="G43" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="H43" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I43" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="J43" s="4"/>
-      <c r="K43" s="4" t="s">
+      <c r="M43" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="L43" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M43" s="4"/>
-      <c r="N43" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="G44" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="H44" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I44" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="J44" s="4"/>
-      <c r="K44" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="L44" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M44" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="N44" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
+      <c r="N43" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <autoFilter ref="A5:N44"/>
   <mergeCells count="3">
@@ -3052,13 +3008,13 @@
     <mergeCell ref="A3:N3"/>
   </mergeCells>
   <conditionalFormatting sqref="N6:N44">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3087,220 +3043,220 @@
   <dimension ref="A1:B30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="B4" s="8" t="n">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$N$6:$N$44,"Pass")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B5" s="8" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$N$6:$N$44,"Fail")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="B6" s="8" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$N$6:$N$44,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="8" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$N$6:$N$44,"Not Run")</f>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="B8" s="7" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B8" s="8" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="B10" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
+      <c r="B10" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$F$6:$F$44,"P1")</f>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$F$6:$F$44,"P2")</f>
         <v>14</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$F$6:$F$44,"P3")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="B14" s="7" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B14" s="8" t="n">
         <f aca="false">SUM(B11:B13)</f>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B17" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Display and default")</f>
         <v>5</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Distribution and rounding (Distribute equally)")</f>
         <v>10</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Selection changes")</f>
         <v>6</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Switching back and saving")</f>
         <v>5</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B21" s="8" t="n">
+      <c r="B21" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Multi-block End Job")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"Work order type coverage")</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="B23" s="8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B23" s="9" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$6:$C$44,"UI and language")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <f aca="false">SUM(B17:B23)</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="B27" s="10"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="B24" s="7" t="n">
-        <f aca="false">SUM(B17:B23)</f>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="s">
-        <v>222</v>
-      </c>
-      <c r="B27" s="9"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="B28" s="9"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="B29" s="9"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="B30" s="9"/>
+      <c r="B28" s="10"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="B29" s="10"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="B30" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3321,162 +3277,161 @@
   <dimension ref="A1:B25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="110"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
+      <c r="B5" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="10" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+      <c r="B6" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="B4" s="11" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="B7" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="B5" s="11" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
+      <c r="B8" s="12" t="s">
         <v>233</v>
       </c>
-      <c r="B6" s="11" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
+      <c r="B9" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="B7" s="11" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
+      <c r="B10" s="12" t="s">
         <v>237</v>
       </c>
-      <c r="B8" s="11" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
+      <c r="B11" s="12" t="s">
         <v>239</v>
       </c>
-      <c r="B9" s="11" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+      <c r="B12" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="B10" s="11" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="B13" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="B11" s="11" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="B12" s="11" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+      <c r="B17" s="13"/>
+    </row>
+    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
         <v>247</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B18" s="13"/>
+    </row>
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+      <c r="B19" s="13"/>
+    </row>
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="B14" s="11" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+      <c r="B23" s="13"/>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
         <v>252</v>
       </c>
-      <c r="B17" s="12"/>
-    </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
-        <v>253</v>
-      </c>
-      <c r="B18" s="12"/>
-    </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
-        <v>254</v>
-      </c>
-      <c r="B19" s="12"/>
-    </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
-        <v>255</v>
-      </c>
-      <c r="B20" s="12"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
-        <v>257</v>
-      </c>
-      <c r="B23" s="12"/>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="s">
-        <v>258</v>
-      </c>
-      <c r="B24" s="12"/>
+      <c r="B24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12" t="s">
-        <v>259</v>
-      </c>
-      <c r="B25" s="12"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>